<commit_message>
added a swaption calibration template for USD
</commit_message>
<xml_diff>
--- a/Calibration Template USD.xlsx
+++ b/Calibration Template USD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/pablo_marchesi_selma_es_ey_com/Documents/Desktop/Calculadoras/Hull-White-Pricer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="8_{00F85499-E803-408C-8FFB-B6A833A2FC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF86FC71-76AA-41B1-A23F-4E7BF040D9C9}"/>
+  <xr:revisionPtr revIDLastSave="312" documentId="8_{00F85499-E803-408C-8FFB-B6A833A2FC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59A869A5-BFA3-45A5-BE59-F5A0B06A7B72}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Curve" sheetId="2" r:id="rId1"/>
@@ -1514,57 +1514,32 @@
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="6"/>
       <c r="B35" s="7"/>
-      <c r="C35" s="13">
-        <f t="shared" si="0"/>
-        <v>125.25277777777778</v>
-      </c>
-      <c r="D35" s="8">
-        <v>0.520305723557551</v>
-      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="8"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="6"/>
       <c r="B36" s="7"/>
-      <c r="C36" s="13">
-        <f t="shared" si="0"/>
-        <v>125.25277777777778</v>
-      </c>
-      <c r="D36" s="8">
-        <v>0.468168168315861</v>
-      </c>
+      <c r="C36" s="13"/>
+      <c r="D36" s="8"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="6"/>
       <c r="B37" s="7"/>
-      <c r="C37" s="13">
-        <f t="shared" si="0"/>
-        <v>125.25277777777778</v>
-      </c>
-      <c r="D37" s="8">
-        <v>0.37848081579099802</v>
-      </c>
+      <c r="C37" s="13"/>
+      <c r="D37" s="8"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="6"/>
       <c r="B38" s="7"/>
-      <c r="C38" s="13">
-        <f t="shared" si="0"/>
-        <v>125.25277777777778</v>
-      </c>
-      <c r="D38" s="8">
-        <v>0.31292981348091498</v>
-      </c>
+      <c r="C38" s="13"/>
+      <c r="D38" s="8"/>
     </row>
     <row r="39" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="9"/>
       <c r="B39" s="10"/>
-      <c r="C39" s="14">
-        <f t="shared" si="0"/>
-        <v>125.25277777777778</v>
-      </c>
-      <c r="D39" s="11">
-        <v>0.26963699121603801</v>
-      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>